<commit_message>
docs: embed polished analytics visualizations into README
</commit_message>
<xml_diff>
--- a/Visuals/FirstSemesterTop50.xlsx
+++ b/Visuals/FirstSemesterTop50.xlsx
@@ -5,12 +5,12 @@
   <workbookPr hidePivotFieldList="1" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fe43dafc9fc930e/Documents/Projects/Data Analysis/Project1_Top 50 Stocks Performance/Dashboard/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4fe43dafc9fc930e/Documents/Projects/Data Analysis/Project1_Top 50 Stocks Performance/Visuals/"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="5" documentId="8_{9726210C-A819-42DB-A36E-4F34425A2CD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3869BD76-E17C-46A7-BD21-F4909B611AAB}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{C7511D92-C801-426A-A780-C8ADC1A9C68B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{C7511D92-C801-426A-A780-C8ADC1A9C68B}"/>
   </bookViews>
   <sheets>
     <sheet name="Pivot Table Data" sheetId="1" r:id="rId1"/>
@@ -9323,7 +9323,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AD3169BA-AB1B-4EB9-94AD-C131BA0C0172}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AD3169BA-AB1B-4EB9-94AD-C131BA0C0172}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="18">
   <location ref="K2:Q14" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="8">
     <pivotField showAll="0"/>

</xml_diff>